<commit_message>
feat(chase): route Scan findings to real owners via author metadata
- adapter.audit_and_persist: resolve per-document owner from author metadata
  (domain/pipeline._resolve_owner) instead of a fixed default; fallback owner
  = nacho (admin escalation) so ownerless docs reach a real inbox.
- scripts/assign_owners.py: stamp corpus author metadata with a realistic name
  embedding the teammate username (augusto/luca/marc/nacho). Idempotent, --check.
- Stamp test_docs/ + demo_corpus/files (45 Office files); leave
  onboarding_procedure_draft.docx deliberately unowned to demo the
  ownerless -> admin escalation path.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/domain/demo_corpus/files/crm_data_dictionary.xlsx
+++ b/domain/demo_corpus/files/crm_data_dictionary.xlsx
@@ -536,7 +536,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -569,7 +568,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -602,7 +600,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -635,7 +632,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -668,7 +664,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -701,7 +696,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -734,7 +728,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>